<commit_message>
Rebuild survey result slides (No.5, No.8) on the group template with Excel-linked charts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UqbJfEc7zNzqZHhWuZQ1kA
</commit_message>
<xml_diff>
--- a/アンケート集計_グラフ.xlsx
+++ b/アンケート集計_グラフ.xlsx
@@ -54,7 +54,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E7D5B"/>
+        <fgColor rgb="00568A80"/>
       </patternFill>
     </fill>
   </fills>
@@ -280,7 +280,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E7D5B"/>
+                <a:srgbClr val="568A80"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -291,7 +291,7 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="C8D6CE"/>
+                <a:srgbClr val="DDD6CC"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -357,7 +357,7 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="F2994A"/>
+              <a:srgbClr val="D0805C"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>

</xml_diff>